<commit_message>
cambios para limitar intensidades horarioa por turno, CAP_PER_INTENSITY en Config, y se usa en select_final_shifts()
</commit_message>
<xml_diff>
--- a/Result/Agents.xlsx
+++ b/Result/Agents.xlsx
@@ -3970,13 +3970,13 @@
         <v>9</v>
       </c>
       <c r="G101" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H101" t="n">
         <v>9</v>
       </c>
       <c r="I101" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J101" t="n">
         <v>0</v>
@@ -4040,13 +4040,13 @@
         <v>9</v>
       </c>
       <c r="G103" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H103" t="n">
         <v>9</v>
       </c>
       <c r="I103" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J103" t="n">
         <v>0</v>
@@ -4075,13 +4075,13 @@
         <v>9</v>
       </c>
       <c r="G104" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H104" t="n">
         <v>9</v>
       </c>
       <c r="I104" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J104" t="n">
         <v>0</v>
@@ -4110,13 +4110,13 @@
         <v>9</v>
       </c>
       <c r="G105" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H105" t="n">
         <v>9</v>
       </c>
       <c r="I105" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J105" t="n">
         <v>0</v>
@@ -4180,13 +4180,13 @@
         <v>9</v>
       </c>
       <c r="G107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H107" t="n">
         <v>9</v>
       </c>
       <c r="I107" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J107" t="n">
         <v>0</v>
@@ -4215,13 +4215,13 @@
         <v>9</v>
       </c>
       <c r="G108" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H108" t="n">
         <v>9</v>
       </c>
       <c r="I108" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J108" t="n">
         <v>0</v>
@@ -4250,13 +4250,13 @@
         <v>9</v>
       </c>
       <c r="G109" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H109" t="n">
         <v>9</v>
       </c>
       <c r="I109" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J109" t="n">
         <v>0</v>
@@ -4285,13 +4285,13 @@
         <v>9</v>
       </c>
       <c r="G110" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H110" t="n">
         <v>9</v>
       </c>
       <c r="I110" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J110" t="n">
         <v>0</v>
@@ -4320,13 +4320,13 @@
         <v>9</v>
       </c>
       <c r="G111" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H111" t="n">
         <v>9</v>
       </c>
       <c r="I111" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J111" t="n">
         <v>0</v>
@@ -4390,13 +4390,13 @@
         <v>9</v>
       </c>
       <c r="G113" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H113" t="n">
         <v>9</v>
       </c>
       <c r="I113" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J113" t="n">
         <v>0</v>
@@ -4425,13 +4425,13 @@
         <v>9</v>
       </c>
       <c r="G114" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H114" t="n">
         <v>9</v>
       </c>
       <c r="I114" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J114" t="n">
         <v>0</v>
@@ -4460,13 +4460,13 @@
         <v>9</v>
       </c>
       <c r="G115" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H115" t="n">
         <v>9</v>
       </c>
       <c r="I115" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J115" t="n">
         <v>0</v>
@@ -4495,13 +4495,13 @@
         <v>9</v>
       </c>
       <c r="G116" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H116" t="n">
         <v>9</v>
       </c>
       <c r="I116" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J116" t="n">
         <v>0</v>
@@ -4530,13 +4530,13 @@
         <v>9</v>
       </c>
       <c r="G117" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H117" t="n">
         <v>9</v>
       </c>
       <c r="I117" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J117" t="n">
         <v>0</v>
@@ -4565,13 +4565,13 @@
         <v>9</v>
       </c>
       <c r="G118" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H118" t="n">
         <v>9</v>
       </c>
       <c r="I118" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J118" t="n">
         <v>0</v>
@@ -4600,13 +4600,13 @@
         <v>9</v>
       </c>
       <c r="G119" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H119" t="n">
         <v>9</v>
       </c>
       <c r="I119" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J119" t="n">
         <v>0</v>
@@ -4635,13 +4635,13 @@
         <v>9</v>
       </c>
       <c r="G120" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H120" t="n">
         <v>9</v>
       </c>
       <c r="I120" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J120" t="n">
         <v>0</v>
@@ -4658,25 +4658,25 @@
         <v>1</v>
       </c>
       <c r="C121" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D121" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E121" t="n">
         <v>9</v>
       </c>
       <c r="F121" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G121" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H121" t="n">
         <v>9</v>
       </c>
       <c r="I121" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J121" t="n">
         <v>0</v>
@@ -4693,25 +4693,25 @@
         <v>1</v>
       </c>
       <c r="C122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D122" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E122" t="n">
         <v>9</v>
       </c>
       <c r="F122" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G122" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H122" t="n">
         <v>9</v>
       </c>
       <c r="I122" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J122" t="n">
         <v>0</v>
@@ -4728,25 +4728,25 @@
         <v>1</v>
       </c>
       <c r="C123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D123" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E123" t="n">
         <v>9</v>
       </c>
       <c r="F123" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G123" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H123" t="n">
         <v>9</v>
       </c>
       <c r="I123" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J123" t="n">
         <v>0</v>
@@ -4798,25 +4798,25 @@
         <v>1</v>
       </c>
       <c r="C125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D125" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E125" t="n">
         <v>9</v>
       </c>
       <c r="F125" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G125" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H125" t="n">
         <v>9</v>
       </c>
       <c r="I125" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J125" t="n">
         <v>0</v>
@@ -4833,25 +4833,25 @@
         <v>1</v>
       </c>
       <c r="C126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D126" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E126" t="n">
         <v>9</v>
       </c>
       <c r="F126" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G126" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H126" t="n">
         <v>9</v>
       </c>
       <c r="I126" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J126" t="n">
         <v>0</v>
@@ -4868,25 +4868,25 @@
         <v>1</v>
       </c>
       <c r="C127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D127" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E127" t="n">
         <v>9</v>
       </c>
       <c r="F127" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G127" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H127" t="n">
         <v>9</v>
       </c>
       <c r="I127" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J127" t="n">
         <v>0</v>
@@ -4903,25 +4903,25 @@
         <v>1</v>
       </c>
       <c r="C128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D128" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E128" t="n">
         <v>9</v>
       </c>
       <c r="F128" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G128" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H128" t="n">
         <v>9</v>
       </c>
       <c r="I128" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J128" t="n">
         <v>0</v>
@@ -4938,22 +4938,22 @@
         <v>1</v>
       </c>
       <c r="C129" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E129" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F129" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G129" t="n">
         <v>8</v>
       </c>
       <c r="H129" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I129" t="n">
         <v>9</v>
@@ -4973,22 +4973,22 @@
         <v>1</v>
       </c>
       <c r="C130" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E130" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F130" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G130" t="n">
         <v>8</v>
       </c>
       <c r="H130" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I130" t="n">
         <v>9</v>
@@ -5008,22 +5008,22 @@
         <v>1</v>
       </c>
       <c r="C131" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D131" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E131" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F131" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G131" t="n">
         <v>8</v>
       </c>
       <c r="H131" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I131" t="n">
         <v>9</v>
@@ -5043,22 +5043,22 @@
         <v>1</v>
       </c>
       <c r="C132" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E132" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F132" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G132" t="n">
         <v>8</v>
       </c>
       <c r="H132" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I132" t="n">
         <v>9</v>
@@ -5078,22 +5078,22 @@
         <v>1</v>
       </c>
       <c r="C133" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D133" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E133" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F133" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G133" t="n">
         <v>8</v>
       </c>
       <c r="H133" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I133" t="n">
         <v>9</v>
@@ -5113,16 +5113,16 @@
         <v>1</v>
       </c>
       <c r="C134" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E134" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F134" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G134" t="n">
         <v>8</v>
@@ -5148,16 +5148,16 @@
         <v>1</v>
       </c>
       <c r="C135" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E135" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F135" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G135" t="n">
         <v>8</v>
@@ -5183,13 +5183,13 @@
         <v>1</v>
       </c>
       <c r="C136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E136" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F136" t="n">
         <v>8</v>
@@ -5988,10 +5988,10 @@
         <v>1</v>
       </c>
       <c r="C159" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D159" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E159" t="n">
         <v>8</v>
@@ -6006,7 +6006,7 @@
         <v>8</v>
       </c>
       <c r="I159" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J159" t="n">
         <v>0</v>
@@ -6058,10 +6058,10 @@
         <v>1</v>
       </c>
       <c r="C161" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D161" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E161" t="n">
         <v>8</v>
@@ -6076,7 +6076,7 @@
         <v>8</v>
       </c>
       <c r="I161" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J161" t="n">
         <v>0</v>
@@ -6093,10 +6093,10 @@
         <v>1</v>
       </c>
       <c r="C162" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D162" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E162" t="n">
         <v>8</v>
@@ -6111,7 +6111,7 @@
         <v>8</v>
       </c>
       <c r="I162" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J162" t="n">
         <v>0</v>
@@ -6128,10 +6128,10 @@
         <v>1</v>
       </c>
       <c r="C163" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D163" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E163" t="n">
         <v>8</v>
@@ -6146,7 +6146,7 @@
         <v>8</v>
       </c>
       <c r="I163" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J163" t="n">
         <v>0</v>
@@ -6163,10 +6163,10 @@
         <v>1</v>
       </c>
       <c r="C164" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D164" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E164" t="n">
         <v>8</v>
@@ -6181,7 +6181,7 @@
         <v>8</v>
       </c>
       <c r="I164" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J164" t="n">
         <v>0</v>
@@ -6198,10 +6198,10 @@
         <v>1</v>
       </c>
       <c r="C165" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D165" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E165" t="n">
         <v>8</v>
@@ -6216,7 +6216,7 @@
         <v>8</v>
       </c>
       <c r="I165" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J165" t="n">
         <v>0</v>
@@ -6233,10 +6233,10 @@
         <v>1</v>
       </c>
       <c r="C166" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D166" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E166" t="n">
         <v>8</v>
@@ -6251,7 +6251,7 @@
         <v>8</v>
       </c>
       <c r="I166" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J166" t="n">
         <v>0</v>
@@ -6268,10 +6268,10 @@
         <v>1</v>
       </c>
       <c r="C167" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D167" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E167" t="n">
         <v>8</v>
@@ -6286,7 +6286,7 @@
         <v>8</v>
       </c>
       <c r="I167" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J167" t="n">
         <v>0</v>
@@ -6303,10 +6303,10 @@
         <v>1</v>
       </c>
       <c r="C168" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D168" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E168" t="n">
         <v>8</v>
@@ -6321,7 +6321,7 @@
         <v>8</v>
       </c>
       <c r="I168" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J168" t="n">
         <v>0</v>
@@ -6338,10 +6338,10 @@
         <v>1</v>
       </c>
       <c r="C169" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D169" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E169" t="n">
         <v>8</v>
@@ -6356,7 +6356,7 @@
         <v>8</v>
       </c>
       <c r="I169" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J169" t="n">
         <v>0</v>
@@ -6408,10 +6408,10 @@
         <v>1</v>
       </c>
       <c r="C171" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D171" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E171" t="n">
         <v>8</v>
@@ -6426,7 +6426,7 @@
         <v>8</v>
       </c>
       <c r="I171" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J171" t="n">
         <v>0</v>
@@ -6478,10 +6478,10 @@
         <v>1</v>
       </c>
       <c r="C173" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D173" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E173" t="n">
         <v>8</v>
@@ -6496,7 +6496,7 @@
         <v>8</v>
       </c>
       <c r="I173" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J173" t="n">
         <v>0</v>
@@ -6513,10 +6513,10 @@
         <v>1</v>
       </c>
       <c r="C174" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D174" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E174" t="n">
         <v>8</v>
@@ -6531,7 +6531,7 @@
         <v>8</v>
       </c>
       <c r="I174" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J174" t="n">
         <v>0</v>
@@ -6548,10 +6548,10 @@
         <v>1</v>
       </c>
       <c r="C175" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D175" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E175" t="n">
         <v>8</v>
@@ -6566,7 +6566,7 @@
         <v>8</v>
       </c>
       <c r="I175" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J175" t="n">
         <v>0</v>
@@ -6583,10 +6583,10 @@
         <v>1</v>
       </c>
       <c r="C176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D176" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E176" t="n">
         <v>8</v>
@@ -6601,7 +6601,7 @@
         <v>8</v>
       </c>
       <c r="I176" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J176" t="n">
         <v>0</v>
@@ -6618,10 +6618,10 @@
         <v>1</v>
       </c>
       <c r="C177" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D177" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E177" t="n">
         <v>8</v>
@@ -6636,7 +6636,7 @@
         <v>8</v>
       </c>
       <c r="I177" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J177" t="n">
         <v>0</v>
@@ -6653,10 +6653,10 @@
         <v>1</v>
       </c>
       <c r="C178" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D178" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E178" t="n">
         <v>8</v>
@@ -6671,7 +6671,7 @@
         <v>8</v>
       </c>
       <c r="I178" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J178" t="n">
         <v>0</v>
@@ -6688,10 +6688,10 @@
         <v>1</v>
       </c>
       <c r="C179" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D179" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E179" t="n">
         <v>8</v>
@@ -6706,7 +6706,7 @@
         <v>8</v>
       </c>
       <c r="I179" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J179" t="n">
         <v>0</v>
@@ -6723,10 +6723,10 @@
         <v>1</v>
       </c>
       <c r="C180" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D180" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E180" t="n">
         <v>8</v>
@@ -6741,7 +6741,7 @@
         <v>8</v>
       </c>
       <c r="I180" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J180" t="n">
         <v>0</v>
@@ -6758,10 +6758,10 @@
         <v>1</v>
       </c>
       <c r="C181" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D181" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E181" t="n">
         <v>8</v>
@@ -6776,7 +6776,7 @@
         <v>8</v>
       </c>
       <c r="I181" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J181" t="n">
         <v>0</v>
@@ -6793,10 +6793,10 @@
         <v>1</v>
       </c>
       <c r="C182" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D182" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E182" t="n">
         <v>8</v>
@@ -6811,7 +6811,7 @@
         <v>8</v>
       </c>
       <c r="I182" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J182" t="n">
         <v>0</v>
@@ -6828,10 +6828,10 @@
         <v>1</v>
       </c>
       <c r="C183" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D183" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E183" t="n">
         <v>8</v>
@@ -6846,7 +6846,7 @@
         <v>8</v>
       </c>
       <c r="I183" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J183" t="n">
         <v>0</v>
@@ -6898,10 +6898,10 @@
         <v>1</v>
       </c>
       <c r="C185" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D185" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E185" t="n">
         <v>8</v>
@@ -6916,7 +6916,7 @@
         <v>8</v>
       </c>
       <c r="I185" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J185" t="n">
         <v>0</v>
@@ -6933,10 +6933,10 @@
         <v>1</v>
       </c>
       <c r="C186" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D186" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E186" t="n">
         <v>8</v>
@@ -6951,7 +6951,7 @@
         <v>8</v>
       </c>
       <c r="I186" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J186" t="n">
         <v>0</v>
@@ -6968,10 +6968,10 @@
         <v>1</v>
       </c>
       <c r="C187" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D187" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E187" t="n">
         <v>8</v>
@@ -6986,7 +6986,7 @@
         <v>8</v>
       </c>
       <c r="I187" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J187" t="n">
         <v>0</v>
@@ -7038,10 +7038,10 @@
         <v>1</v>
       </c>
       <c r="C189" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D189" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E189" t="n">
         <v>8</v>
@@ -7056,7 +7056,7 @@
         <v>8</v>
       </c>
       <c r="I189" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J189" t="n">
         <v>0</v>
@@ -7073,10 +7073,10 @@
         <v>1</v>
       </c>
       <c r="C190" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D190" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E190" t="n">
         <v>8</v>
@@ -7091,7 +7091,7 @@
         <v>8</v>
       </c>
       <c r="I190" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J190" t="n">
         <v>0</v>
@@ -7108,10 +7108,10 @@
         <v>1</v>
       </c>
       <c r="C191" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D191" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E191" t="n">
         <v>8</v>
@@ -7126,7 +7126,7 @@
         <v>8</v>
       </c>
       <c r="I191" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J191" t="n">
         <v>0</v>
@@ -7143,10 +7143,10 @@
         <v>1</v>
       </c>
       <c r="C192" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D192" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E192" t="n">
         <v>8</v>
@@ -7161,7 +7161,7 @@
         <v>8</v>
       </c>
       <c r="I192" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J192" t="n">
         <v>0</v>
@@ -7178,10 +7178,10 @@
         <v>1</v>
       </c>
       <c r="C193" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D193" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E193" t="n">
         <v>8</v>
@@ -7196,7 +7196,7 @@
         <v>8</v>
       </c>
       <c r="I193" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J193" t="n">
         <v>0</v>
@@ -7213,10 +7213,10 @@
         <v>1</v>
       </c>
       <c r="C194" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D194" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E194" t="n">
         <v>8</v>
@@ -7231,7 +7231,7 @@
         <v>8</v>
       </c>
       <c r="I194" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J194" t="n">
         <v>0</v>
@@ -8088,10 +8088,10 @@
         <v>1</v>
       </c>
       <c r="C219" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D219" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E219" t="n">
         <v>8</v>
@@ -8100,7 +8100,7 @@
         <v>8</v>
       </c>
       <c r="G219" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H219" t="n">
         <v>8</v>
@@ -8123,10 +8123,10 @@
         <v>1</v>
       </c>
       <c r="C220" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D220" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E220" t="n">
         <v>8</v>
@@ -8135,7 +8135,7 @@
         <v>8</v>
       </c>
       <c r="G220" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H220" t="n">
         <v>8</v>
@@ -8158,10 +8158,10 @@
         <v>1</v>
       </c>
       <c r="C221" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D221" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E221" t="n">
         <v>8</v>
@@ -8170,7 +8170,7 @@
         <v>8</v>
       </c>
       <c r="G221" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H221" t="n">
         <v>8</v>
@@ -8193,10 +8193,10 @@
         <v>1</v>
       </c>
       <c r="C222" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D222" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E222" t="n">
         <v>8</v>
@@ -8205,7 +8205,7 @@
         <v>8</v>
       </c>
       <c r="G222" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H222" t="n">
         <v>8</v>
@@ -12463,10 +12463,10 @@
         <v>1</v>
       </c>
       <c r="C344" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D344" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E344" t="n">
         <v>9</v>
@@ -12481,7 +12481,7 @@
         <v>8</v>
       </c>
       <c r="I344" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J344" t="n">
         <v>0</v>
@@ -12498,10 +12498,10 @@
         <v>1</v>
       </c>
       <c r="C345" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D345" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E345" t="n">
         <v>9</v>
@@ -12516,7 +12516,7 @@
         <v>8</v>
       </c>
       <c r="I345" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J345" t="n">
         <v>0</v>
@@ -12533,10 +12533,10 @@
         <v>1</v>
       </c>
       <c r="C346" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D346" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E346" t="n">
         <v>9</v>
@@ -12551,7 +12551,7 @@
         <v>8</v>
       </c>
       <c r="I346" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J346" t="n">
         <v>0</v>
@@ -12603,10 +12603,10 @@
         <v>1</v>
       </c>
       <c r="C348" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D348" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E348" t="n">
         <v>9</v>
@@ -12621,7 +12621,7 @@
         <v>8</v>
       </c>
       <c r="I348" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J348" t="n">
         <v>0</v>
@@ -12638,10 +12638,10 @@
         <v>1</v>
       </c>
       <c r="C349" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D349" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E349" t="n">
         <v>9</v>
@@ -12656,7 +12656,7 @@
         <v>8</v>
       </c>
       <c r="I349" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J349" t="n">
         <v>0</v>
@@ -12708,10 +12708,10 @@
         <v>1</v>
       </c>
       <c r="C351" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D351" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E351" t="n">
         <v>9</v>
@@ -12726,7 +12726,7 @@
         <v>8</v>
       </c>
       <c r="I351" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J351" t="n">
         <v>0</v>
@@ -12743,10 +12743,10 @@
         <v>1</v>
       </c>
       <c r="C352" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D352" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E352" t="n">
         <v>9</v>
@@ -12761,7 +12761,7 @@
         <v>8</v>
       </c>
       <c r="I352" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J352" t="n">
         <v>0</v>
@@ -12778,10 +12778,10 @@
         <v>1</v>
       </c>
       <c r="C353" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D353" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E353" t="n">
         <v>9</v>
@@ -12796,7 +12796,7 @@
         <v>8</v>
       </c>
       <c r="I353" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J353" t="n">
         <v>0</v>
@@ -12813,10 +12813,10 @@
         <v>1</v>
       </c>
       <c r="C354" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D354" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E354" t="n">
         <v>9</v>
@@ -12831,7 +12831,7 @@
         <v>8</v>
       </c>
       <c r="I354" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J354" t="n">
         <v>0</v>
@@ -12918,10 +12918,10 @@
         <v>1</v>
       </c>
       <c r="C357" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D357" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E357" t="n">
         <v>9</v>
@@ -12930,7 +12930,7 @@
         <v>9</v>
       </c>
       <c r="G357" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H357" t="n">
         <v>8</v>
@@ -12953,10 +12953,10 @@
         <v>1</v>
       </c>
       <c r="C358" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D358" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E358" t="n">
         <v>9</v>
@@ -12965,7 +12965,7 @@
         <v>9</v>
       </c>
       <c r="G358" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H358" t="n">
         <v>8</v>
@@ -12988,10 +12988,10 @@
         <v>1</v>
       </c>
       <c r="C359" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D359" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E359" t="n">
         <v>9</v>
@@ -13000,7 +13000,7 @@
         <v>9</v>
       </c>
       <c r="G359" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H359" t="n">
         <v>8</v>
@@ -13023,10 +13023,10 @@
         <v>1</v>
       </c>
       <c r="C360" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D360" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E360" t="n">
         <v>9</v>
@@ -13035,7 +13035,7 @@
         <v>9</v>
       </c>
       <c r="G360" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H360" t="n">
         <v>8</v>

</xml_diff>

<commit_message>
Fix for agent reordering; heterogeneous works best.
</commit_message>
<xml_diff>
--- a/Result/Agents.xlsx
+++ b/Result/Agents.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pruebas\Proyect_WFM\Result\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBBBED1-DC16-42F7-9275-43F73F7041F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20637404-7422-4141-AEC8-B495B8CF9127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -133,8 +133,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1393,7 +1394,7 @@
       <c r="Q17">
         <v>0</v>
       </c>
-      <c r="R17">
+      <c r="R17" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>